<commit_message>
UI enhancements: fonts, particles background, Lottie loader, accessibility improvements
</commit_message>
<xml_diff>
--- a/data/students.xlsx
+++ b/data/students.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="h:\Users\Asus\Desktop\oat\J.A.R.V.I.S\Excel_Agent\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AC3E57C-6605-4012-B50C-29045E5BC2D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55225DCE-F6C4-4B11-BC81-7FDEB48AE948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="48">
   <si>
     <t>students</t>
   </si>
@@ -137,6 +137,33 @@
   </si>
   <si>
     <t>๐๙๖-๑๕๓๙๕๑๔</t>
+  </si>
+  <si>
+    <t>ยศวัช</t>
+  </si>
+  <si>
+    <t>เรืองศรี</t>
+  </si>
+  <si>
+    <t>ลูกแถว มว.๓ หมู่ ๒</t>
+  </si>
+  <si>
+    <t>๐๙๓-๕๓๑-๕๑๕๕</t>
+  </si>
+  <si>
+    <t>สุวิจักขณ์</t>
+  </si>
+  <si>
+    <t>วย.</t>
+  </si>
+  <si>
+    <t>หน.มว.๑ หมู่ ๒</t>
+  </si>
+  <si>
+    <t>พัน.๒ ร้อย.๒</t>
+  </si>
+  <si>
+    <t>๐๙๑-๗๑๖๖๙๙๔</t>
   </si>
 </sst>
 </file>
@@ -191,9 +218,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="59" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -501,7 +531,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -515,30 +545,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="28.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
     </row>
     <row r="2" spans="1:10" ht="21" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
     </row>
     <row r="3" spans="1:10" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -691,6 +721,336 @@
         <v>38</v>
       </c>
       <c r="J7" s="1"/>
+    </row>
+    <row r="8" spans="1:10" ht="21" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>106</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="2">
+        <v>5</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J8" s="1"/>
+    </row>
+    <row r="9" spans="1:10" ht="21" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>54</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" s="2">
+        <v>5</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J9" s="1"/>
+    </row>
+    <row r="10" spans="1:10" ht="21" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>999</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="2">
+        <v>3</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="J10" s="1"/>
+    </row>
+    <row r="11" spans="1:10" ht="21" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>1051</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" s="2">
+        <v>5</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="J11" s="1"/>
+    </row>
+    <row r="12" spans="1:10" ht="21" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>106</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="2">
+        <v>5</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="1:10" ht="21" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>54</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="2">
+        <v>5</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:10" ht="21" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>999</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="2">
+        <v>3</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="J14" s="1"/>
+    </row>
+    <row r="15" spans="1:10" ht="21" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>1051</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="2">
+        <v>5</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="J15" s="1"/>
+    </row>
+    <row r="16" spans="1:10" ht="21" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>54</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="2">
+        <v>5</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J16" s="1"/>
+    </row>
+    <row r="17" spans="1:10" ht="21" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>999</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" s="2">
+        <v>3</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="1:10" ht="21" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>1051</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E18" s="2">
+        <v>5</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="J18" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>